<commit_message>
scout line 색깔 변경
</commit_message>
<xml_diff>
--- a/뷰어 샘플 개발 일정표_윤은지_250916.xlsx
+++ b/뷰어 샘플 개발 일정표_윤은지_250916.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\sample\2\Qt3DViewer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62E9AC98-041E-490F-9DB5-6DA2D691FFC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74504FA8-C6EA-4BBE-9B7F-05D2ADDF3FD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="420" yWindow="2670" windowWidth="56160" windowHeight="23850" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-2325" yWindow="2205" windowWidth="56160" windowHeight="23850" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Viewer 샘플" sheetId="8" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="63">
   <si>
     <t>구 분</t>
     <phoneticPr fontId="3" type="noConversion"/>
@@ -4786,11 +4786,13 @@
       <c r="Y38" s="87"/>
       <c r="Z38" s="87"/>
       <c r="AA38" s="89"/>
-      <c r="AB38" s="12"/>
-      <c r="AC38" s="13"/>
-      <c r="AD38" s="13"/>
-      <c r="AE38" s="13"/>
-      <c r="AF38" s="14"/>
+      <c r="AB38" s="86"/>
+      <c r="AC38" s="87"/>
+      <c r="AD38" s="87"/>
+      <c r="AE38" s="87"/>
+      <c r="AF38" s="89" t="s">
+        <v>43</v>
+      </c>
       <c r="AG38" s="12"/>
       <c r="AH38" s="12"/>
       <c r="AI38" s="13"/>
@@ -4960,11 +4962,11 @@
       <c r="T41" s="18"/>
       <c r="U41" s="25"/>
       <c r="V41" s="26"/>
-      <c r="W41" s="21"/>
-      <c r="X41" s="21"/>
-      <c r="Y41" s="18"/>
-      <c r="Z41" s="18"/>
-      <c r="AA41" s="26"/>
+      <c r="W41" s="86"/>
+      <c r="X41" s="86"/>
+      <c r="Y41" s="87"/>
+      <c r="Z41" s="87"/>
+      <c r="AA41" s="89"/>
       <c r="AB41" s="21"/>
       <c r="AC41" s="18"/>
       <c r="AD41" s="18"/>
@@ -5080,11 +5082,11 @@
       <c r="T43" s="18"/>
       <c r="U43" s="25"/>
       <c r="V43" s="26"/>
-      <c r="W43" s="21"/>
-      <c r="X43" s="21"/>
-      <c r="Y43" s="18"/>
-      <c r="Z43" s="18"/>
-      <c r="AA43" s="26"/>
+      <c r="W43" s="86"/>
+      <c r="X43" s="86"/>
+      <c r="Y43" s="87"/>
+      <c r="Z43" s="87"/>
+      <c r="AA43" s="89"/>
       <c r="AB43" s="21"/>
       <c r="AC43" s="18"/>
       <c r="AD43" s="18"/>

</xml_diff>

<commit_message>
scout line 동기화 완료
</commit_message>
<xml_diff>
--- a/뷰어 샘플 개발 일정표_윤은지_250916.xlsx
+++ b/뷰어 샘플 개발 일정표_윤은지_250916.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\sample\2\Qt3DViewer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74504FA8-C6EA-4BBE-9B7F-05D2ADDF3FD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D79FCA85-36AB-4C66-BEB5-B2B9E432D6B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-2325" yWindow="2205" windowWidth="56160" windowHeight="23850" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="2205" windowWidth="51180" windowHeight="23850" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Viewer 샘플" sheetId="8" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="64">
   <si>
     <t>구 분</t>
     <phoneticPr fontId="3" type="noConversion"/>
@@ -274,6 +274,10 @@
   </si>
   <si>
     <t>MPR 3뷰 출력</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>10월 22일</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -1442,7 +1446,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1713,6 +1717,24 @@
     <xf numFmtId="0" fontId="5" fillId="30" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="28" fillId="27" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1722,22 +1744,16 @@
     <xf numFmtId="0" fontId="28" fillId="27" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="30" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="30" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="25" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="30" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="25" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="25" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="25" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="30" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2504,11 +2520,11 @@
       <c r="BY2" s="27"/>
     </row>
     <row r="3" spans="1:78" s="2" customFormat="1" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B3" s="93" t="s">
+      <c r="B3" s="90" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="95"/>
-      <c r="D3" s="96"/>
+      <c r="C3" s="92"/>
+      <c r="D3" s="93"/>
       <c r="E3" s="69"/>
       <c r="F3" s="72" t="s">
         <v>4</v>
@@ -2603,9 +2619,9 @@
       <c r="BZ3" s="3"/>
     </row>
     <row r="4" spans="1:78" s="2" customFormat="1" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B4" s="94"/>
-      <c r="C4" s="97"/>
-      <c r="D4" s="98"/>
+      <c r="B4" s="91"/>
+      <c r="C4" s="94"/>
+      <c r="D4" s="95"/>
       <c r="E4" s="70"/>
       <c r="F4" s="71">
         <v>1</v>
@@ -2772,7 +2788,7 @@
       <c r="C5" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="90" t="s">
+      <c r="D5" s="96" t="s">
         <v>19</v>
       </c>
       <c r="E5" s="54" t="s">
@@ -2833,7 +2849,7 @@
     <row r="6" spans="1:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B6" s="17"/>
       <c r="C6" s="40"/>
-      <c r="D6" s="91"/>
+      <c r="D6" s="97"/>
       <c r="E6" s="55" t="s">
         <v>34</v>
       </c>
@@ -2892,7 +2908,7 @@
     <row r="7" spans="1:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B7" s="17"/>
       <c r="C7" s="40"/>
-      <c r="D7" s="90" t="s">
+      <c r="D7" s="96" t="s">
         <v>20</v>
       </c>
       <c r="E7" s="54" t="s">
@@ -2953,7 +2969,7 @@
     <row r="8" spans="1:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B8" s="17"/>
       <c r="C8" s="40"/>
-      <c r="D8" s="91"/>
+      <c r="D8" s="97"/>
       <c r="E8" s="55" t="s">
         <v>34</v>
       </c>
@@ -3012,7 +3028,7 @@
     <row r="9" spans="1:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B9" s="17"/>
       <c r="C9" s="40"/>
-      <c r="D9" s="90" t="s">
+      <c r="D9" s="96" t="s">
         <v>22</v>
       </c>
       <c r="E9" s="54" t="s">
@@ -3073,7 +3089,7 @@
     <row r="10" spans="1:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B10" s="17"/>
       <c r="C10" s="40"/>
-      <c r="D10" s="91"/>
+      <c r="D10" s="97"/>
       <c r="E10" s="55" t="s">
         <v>34</v>
       </c>
@@ -3132,7 +3148,7 @@
     <row r="11" spans="1:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B11" s="17"/>
       <c r="C11" s="40"/>
-      <c r="D11" s="90" t="s">
+      <c r="D11" s="96" t="s">
         <v>23</v>
       </c>
       <c r="E11" s="54" t="s">
@@ -3193,7 +3209,7 @@
     <row r="12" spans="1:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B12" s="17"/>
       <c r="C12" s="40"/>
-      <c r="D12" s="91"/>
+      <c r="D12" s="97"/>
       <c r="E12" s="55" t="s">
         <v>34</v>
       </c>
@@ -3252,7 +3268,7 @@
     <row r="13" spans="1:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B13" s="17"/>
       <c r="C13" s="40"/>
-      <c r="D13" s="90" t="s">
+      <c r="D13" s="96" t="s">
         <v>21</v>
       </c>
       <c r="E13" s="54" t="s">
@@ -3313,7 +3329,7 @@
     <row r="14" spans="1:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B14" s="17"/>
       <c r="C14" s="40"/>
-      <c r="D14" s="91"/>
+      <c r="D14" s="97"/>
       <c r="E14" s="61" t="s">
         <v>34</v>
       </c>
@@ -3374,7 +3390,7 @@
       <c r="C15" s="40" t="s">
         <v>14</v>
       </c>
-      <c r="D15" s="90" t="s">
+      <c r="D15" s="96" t="s">
         <v>24</v>
       </c>
       <c r="E15" s="54" t="s">
@@ -3435,7 +3451,7 @@
     <row r="16" spans="1:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B16" s="17"/>
       <c r="C16" s="40"/>
-      <c r="D16" s="91"/>
+      <c r="D16" s="97"/>
       <c r="E16" s="55" t="s">
         <v>34</v>
       </c>
@@ -3494,7 +3510,7 @@
     <row r="17" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B17" s="17"/>
       <c r="C17" s="40"/>
-      <c r="D17" s="90" t="s">
+      <c r="D17" s="96" t="s">
         <v>25</v>
       </c>
       <c r="E17" s="60" t="s">
@@ -3555,7 +3571,7 @@
     <row r="18" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B18" s="17"/>
       <c r="C18" s="40"/>
-      <c r="D18" s="91"/>
+      <c r="D18" s="97"/>
       <c r="E18" s="61" t="s">
         <v>34</v>
       </c>
@@ -3616,7 +3632,7 @@
       <c r="C19" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="D19" s="90" t="s">
+      <c r="D19" s="96" t="s">
         <v>26</v>
       </c>
       <c r="E19" s="54" t="s">
@@ -3677,7 +3693,7 @@
     <row r="20" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B20" s="17"/>
       <c r="C20" s="40"/>
-      <c r="D20" s="91"/>
+      <c r="D20" s="97"/>
       <c r="E20" s="55" t="s">
         <v>34</v>
       </c>
@@ -3736,7 +3752,7 @@
     <row r="21" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B21" s="17"/>
       <c r="C21" s="40"/>
-      <c r="D21" s="90" t="s">
+      <c r="D21" s="96" t="s">
         <v>27</v>
       </c>
       <c r="E21" s="60" t="s">
@@ -3797,7 +3813,7 @@
     <row r="22" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B22" s="17"/>
       <c r="C22" s="40"/>
-      <c r="D22" s="91"/>
+      <c r="D22" s="97"/>
       <c r="E22" s="61" t="s">
         <v>34</v>
       </c>
@@ -3858,7 +3874,7 @@
       <c r="C23" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="90" t="s">
+      <c r="D23" s="96" t="s">
         <v>28</v>
       </c>
       <c r="E23" s="54" t="s">
@@ -3919,7 +3935,7 @@
     <row r="24" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B24" s="17"/>
       <c r="C24" s="40"/>
-      <c r="D24" s="91"/>
+      <c r="D24" s="97"/>
       <c r="E24" s="55" t="s">
         <v>34</v>
       </c>
@@ -3978,7 +3994,7 @@
     <row r="25" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B25" s="17"/>
       <c r="C25" s="40"/>
-      <c r="D25" s="90" t="s">
+      <c r="D25" s="96" t="s">
         <v>29</v>
       </c>
       <c r="E25" s="54" t="s">
@@ -4039,7 +4055,7 @@
     <row r="26" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B26" s="17"/>
       <c r="C26" s="40"/>
-      <c r="D26" s="91"/>
+      <c r="D26" s="97"/>
       <c r="E26" s="55" t="s">
         <v>34</v>
       </c>
@@ -4098,7 +4114,7 @@
     <row r="27" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B27" s="17"/>
       <c r="C27" s="40"/>
-      <c r="D27" s="90" t="s">
+      <c r="D27" s="96" t="s">
         <v>30</v>
       </c>
       <c r="E27" s="60" t="s">
@@ -4159,7 +4175,7 @@
     <row r="28" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B28" s="17"/>
       <c r="C28" s="40"/>
-      <c r="D28" s="91"/>
+      <c r="D28" s="97"/>
       <c r="E28" s="61" t="s">
         <v>34</v>
       </c>
@@ -4220,7 +4236,7 @@
       <c r="C29" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="D29" s="90" t="s">
+      <c r="D29" s="96" t="s">
         <v>32</v>
       </c>
       <c r="E29" s="54" t="s">
@@ -4281,7 +4297,7 @@
     <row r="30" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B30" s="17"/>
       <c r="C30" s="40"/>
-      <c r="D30" s="91"/>
+      <c r="D30" s="97"/>
       <c r="E30" s="55" t="s">
         <v>34</v>
       </c>
@@ -4340,7 +4356,7 @@
     <row r="31" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B31" s="17"/>
       <c r="C31" s="40"/>
-      <c r="D31" s="90" t="s">
+      <c r="D31" s="96" t="s">
         <v>60</v>
       </c>
       <c r="E31" s="54" t="s">
@@ -4401,7 +4417,7 @@
     <row r="32" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B32" s="17"/>
       <c r="C32" s="40"/>
-      <c r="D32" s="91"/>
+      <c r="D32" s="97"/>
       <c r="E32" s="55" t="s">
         <v>34</v>
       </c>
@@ -4460,7 +4476,7 @@
     <row r="33" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B33" s="17"/>
       <c r="C33" s="40"/>
-      <c r="D33" s="90" t="s">
+      <c r="D33" s="96" t="s">
         <v>31</v>
       </c>
       <c r="E33" s="54" t="s">
@@ -4521,7 +4537,7 @@
     <row r="34" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B34" s="17"/>
       <c r="C34" s="40"/>
-      <c r="D34" s="91"/>
+      <c r="D34" s="97"/>
       <c r="E34" s="55" t="s">
         <v>34</v>
       </c>
@@ -4580,7 +4596,7 @@
     <row r="35" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B35" s="17"/>
       <c r="C35" s="40"/>
-      <c r="D35" s="90" t="s">
+      <c r="D35" s="96" t="s">
         <v>62</v>
       </c>
       <c r="E35" s="54" t="s">
@@ -4641,7 +4657,7 @@
     <row r="36" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B36" s="17"/>
       <c r="C36" s="40"/>
-      <c r="D36" s="91"/>
+      <c r="D36" s="97"/>
       <c r="E36" s="55" t="s">
         <v>34</v>
       </c>
@@ -4700,7 +4716,7 @@
     <row r="37" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B37" s="17"/>
       <c r="C37" s="40"/>
-      <c r="D37" s="90" t="s">
+      <c r="D37" s="96" t="s">
         <v>57</v>
       </c>
       <c r="E37" s="60" t="s">
@@ -4760,7 +4776,7 @@
     <row r="38" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B38" s="17"/>
       <c r="C38" s="40"/>
-      <c r="D38" s="91"/>
+      <c r="D38" s="97"/>
       <c r="E38" s="61" t="s">
         <v>34</v>
       </c>
@@ -4821,7 +4837,7 @@
       <c r="C39" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="D39" s="90" t="s">
+      <c r="D39" s="96" t="s">
         <v>54</v>
       </c>
       <c r="E39" s="60" t="s">
@@ -4884,7 +4900,7 @@
     <row r="40" spans="2:78" ht="22.15" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B40" s="17"/>
       <c r="C40" s="40"/>
-      <c r="D40" s="92"/>
+      <c r="D40" s="98"/>
       <c r="E40" s="62" t="s">
         <v>34</v>
       </c>
@@ -4941,7 +4957,7 @@
     <row r="41" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B41" s="17"/>
       <c r="C41" s="40"/>
-      <c r="D41" s="91"/>
+      <c r="D41" s="97"/>
       <c r="E41" s="61" t="s">
         <v>34</v>
       </c>
@@ -4967,26 +4983,28 @@
       <c r="Y41" s="87"/>
       <c r="Z41" s="87"/>
       <c r="AA41" s="89"/>
-      <c r="AB41" s="21"/>
-      <c r="AC41" s="18"/>
-      <c r="AD41" s="18"/>
-      <c r="AE41" s="18"/>
-      <c r="AF41" s="26"/>
-      <c r="AG41" s="73"/>
-      <c r="AH41" s="73"/>
-      <c r="AI41" s="74"/>
-      <c r="AJ41" s="74"/>
-      <c r="AK41" s="75"/>
-      <c r="AL41" s="73"/>
-      <c r="AM41" s="74"/>
-      <c r="AN41" s="74"/>
-      <c r="AO41" s="76"/>
-      <c r="AP41" s="75"/>
-      <c r="AQ41" s="21"/>
-      <c r="AR41" s="21"/>
-      <c r="AS41" s="18"/>
-      <c r="AT41" s="18"/>
-      <c r="AU41" s="26"/>
+      <c r="AB41" s="86"/>
+      <c r="AC41" s="87"/>
+      <c r="AD41" s="87"/>
+      <c r="AE41" s="87"/>
+      <c r="AF41" s="89"/>
+      <c r="AG41" s="99"/>
+      <c r="AH41" s="99"/>
+      <c r="AI41" s="100"/>
+      <c r="AJ41" s="100"/>
+      <c r="AK41" s="101"/>
+      <c r="AL41" s="99"/>
+      <c r="AM41" s="100"/>
+      <c r="AN41" s="100"/>
+      <c r="AO41" s="102"/>
+      <c r="AP41" s="101"/>
+      <c r="AQ41" s="86"/>
+      <c r="AR41" s="86"/>
+      <c r="AS41" s="87"/>
+      <c r="AT41" s="87"/>
+      <c r="AU41" s="89" t="s">
+        <v>63</v>
+      </c>
       <c r="AY41" s="3"/>
       <c r="BD41" s="3"/>
       <c r="BH41" s="3"/>
@@ -4998,7 +5016,7 @@
     <row r="42" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B42" s="17"/>
       <c r="C42" s="40"/>
-      <c r="D42" s="90" t="s">
+      <c r="D42" s="96" t="s">
         <v>45</v>
       </c>
       <c r="E42" s="60" t="s">
@@ -5061,7 +5079,7 @@
     <row r="43" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B43" s="17"/>
       <c r="C43" s="40"/>
-      <c r="D43" s="91"/>
+      <c r="D43" s="97"/>
       <c r="E43" s="62" t="s">
         <v>34</v>
       </c>
@@ -5087,26 +5105,28 @@
       <c r="Y43" s="87"/>
       <c r="Z43" s="87"/>
       <c r="AA43" s="89"/>
-      <c r="AB43" s="21"/>
-      <c r="AC43" s="18"/>
-      <c r="AD43" s="18"/>
-      <c r="AE43" s="18"/>
-      <c r="AF43" s="26"/>
-      <c r="AG43" s="21"/>
-      <c r="AH43" s="21"/>
-      <c r="AI43" s="18"/>
-      <c r="AJ43" s="18"/>
-      <c r="AK43" s="26"/>
-      <c r="AL43" s="21"/>
-      <c r="AM43" s="18"/>
-      <c r="AN43" s="18"/>
-      <c r="AO43" s="25"/>
-      <c r="AP43" s="26"/>
-      <c r="AQ43" s="21"/>
-      <c r="AR43" s="18"/>
-      <c r="AS43" s="18"/>
-      <c r="AT43" s="18"/>
-      <c r="AU43" s="26"/>
+      <c r="AB43" s="86"/>
+      <c r="AC43" s="87"/>
+      <c r="AD43" s="87"/>
+      <c r="AE43" s="87"/>
+      <c r="AF43" s="89"/>
+      <c r="AG43" s="86"/>
+      <c r="AH43" s="86"/>
+      <c r="AI43" s="87"/>
+      <c r="AJ43" s="87"/>
+      <c r="AK43" s="89"/>
+      <c r="AL43" s="86"/>
+      <c r="AM43" s="87"/>
+      <c r="AN43" s="87"/>
+      <c r="AO43" s="88"/>
+      <c r="AP43" s="89"/>
+      <c r="AQ43" s="86"/>
+      <c r="AR43" s="87"/>
+      <c r="AS43" s="87"/>
+      <c r="AT43" s="87"/>
+      <c r="AU43" s="89" t="s">
+        <v>63</v>
+      </c>
       <c r="AY43" s="3"/>
       <c r="BD43" s="3"/>
       <c r="BH43" s="3"/>
@@ -5118,7 +5138,7 @@
     <row r="44" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B44" s="17"/>
       <c r="C44" s="40"/>
-      <c r="D44" s="90" t="s">
+      <c r="D44" s="96" t="s">
         <v>46</v>
       </c>
       <c r="E44" s="60" t="s">
@@ -5179,7 +5199,7 @@
     <row r="45" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B45" s="17"/>
       <c r="C45" s="40"/>
-      <c r="D45" s="91"/>
+      <c r="D45" s="97"/>
       <c r="E45" s="62" t="s">
         <v>34</v>
       </c>
@@ -5236,7 +5256,7 @@
     <row r="46" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B46" s="17"/>
       <c r="C46" s="40"/>
-      <c r="D46" s="90" t="s">
+      <c r="D46" s="96" t="s">
         <v>47</v>
       </c>
       <c r="E46" s="60" t="s">
@@ -5297,7 +5317,7 @@
     <row r="47" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B47" s="17"/>
       <c r="C47" s="40"/>
-      <c r="D47" s="91"/>
+      <c r="D47" s="97"/>
       <c r="E47" s="62" t="s">
         <v>34</v>
       </c>
@@ -5354,7 +5374,7 @@
     <row r="48" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B48" s="17"/>
       <c r="C48" s="40"/>
-      <c r="D48" s="90" t="s">
+      <c r="D48" s="96" t="s">
         <v>48</v>
       </c>
       <c r="E48" s="60" t="s">
@@ -5415,7 +5435,7 @@
     <row r="49" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B49" s="17"/>
       <c r="C49" s="40"/>
-      <c r="D49" s="91"/>
+      <c r="D49" s="97"/>
       <c r="E49" s="62" t="s">
         <v>34</v>
       </c>
@@ -5472,7 +5492,7 @@
     <row r="50" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B50" s="17"/>
       <c r="C50" s="40"/>
-      <c r="D50" s="90" t="s">
+      <c r="D50" s="96" t="s">
         <v>49</v>
       </c>
       <c r="E50" s="60" t="s">
@@ -5533,7 +5553,7 @@
     <row r="51" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B51" s="17"/>
       <c r="C51" s="40"/>
-      <c r="D51" s="91"/>
+      <c r="D51" s="97"/>
       <c r="E51" s="62" t="s">
         <v>34</v>
       </c>
@@ -5590,7 +5610,7 @@
     <row r="52" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B52" s="17"/>
       <c r="C52" s="40"/>
-      <c r="D52" s="90" t="s">
+      <c r="D52" s="96" t="s">
         <v>50</v>
       </c>
       <c r="E52" s="60" t="s">
@@ -5651,7 +5671,7 @@
     <row r="53" spans="2:78" ht="22.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B53" s="17"/>
       <c r="C53" s="40"/>
-      <c r="D53" s="91"/>
+      <c r="D53" s="97"/>
       <c r="E53" s="62" t="s">
         <v>34</v>
       </c>
@@ -8481,6 +8501,16 @@
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="D33:D34"/>
+    <mergeCell ref="D37:D38"/>
+    <mergeCell ref="D39:D41"/>
+    <mergeCell ref="D52:D53"/>
+    <mergeCell ref="D42:D43"/>
+    <mergeCell ref="D44:D45"/>
+    <mergeCell ref="D46:D47"/>
+    <mergeCell ref="D48:D49"/>
+    <mergeCell ref="D50:D51"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="C3:D4"/>
     <mergeCell ref="D35:D36"/>
@@ -8497,16 +8527,6 @@
     <mergeCell ref="D25:D26"/>
     <mergeCell ref="D27:D28"/>
     <mergeCell ref="D29:D30"/>
-    <mergeCell ref="D31:D32"/>
-    <mergeCell ref="D33:D34"/>
-    <mergeCell ref="D37:D38"/>
-    <mergeCell ref="D39:D41"/>
-    <mergeCell ref="D52:D53"/>
-    <mergeCell ref="D42:D43"/>
-    <mergeCell ref="D44:D45"/>
-    <mergeCell ref="D46:D47"/>
-    <mergeCell ref="D48:D49"/>
-    <mergeCell ref="D50:D51"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>

<commit_message>
볼륨 - scout line 연동
</commit_message>
<xml_diff>
--- a/뷰어 샘플 개발 일정표_윤은지_250916.xlsx
+++ b/뷰어 샘플 개발 일정표_윤은지_250916.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\sample\2\Qt3DViewer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D1056BD-9380-44A3-887C-97C1E55549FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B366903-AFC7-4849-A682-4A3F9BE6A0FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8700" yWindow="3990" windowWidth="39510" windowHeight="21540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8700" yWindow="3990" windowWidth="34935" windowHeight="21540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Viewer 샘플" sheetId="8" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="71">
   <si>
     <t>구 분</t>
     <phoneticPr fontId="3" type="noConversion"/>
@@ -302,6 +302,10 @@
   </si>
   <si>
     <t>11월 28일</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>11월 19일</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -5858,11 +5862,13 @@
       <c r="AN55" s="88"/>
       <c r="AO55" s="88"/>
       <c r="AP55" s="86"/>
-      <c r="AQ55" s="21"/>
-      <c r="AR55" s="18"/>
-      <c r="AS55" s="18"/>
-      <c r="AT55" s="18"/>
-      <c r="AU55" s="26"/>
+      <c r="AQ55" s="87"/>
+      <c r="AR55" s="88"/>
+      <c r="AS55" s="88"/>
+      <c r="AT55" s="88"/>
+      <c r="AU55" s="79" t="s">
+        <v>70</v>
+      </c>
       <c r="AY55" s="3"/>
       <c r="BD55" s="3"/>
       <c r="BH55" s="3"/>
@@ -5971,16 +5977,18 @@
       <c r="AI57" s="13"/>
       <c r="AJ57" s="13"/>
       <c r="AK57" s="14"/>
-      <c r="AL57" s="21"/>
-      <c r="AM57" s="18"/>
-      <c r="AN57" s="18"/>
-      <c r="AO57" s="25"/>
-      <c r="AP57" s="26"/>
-      <c r="AQ57" s="21"/>
-      <c r="AR57" s="18"/>
-      <c r="AS57" s="18"/>
-      <c r="AT57" s="18"/>
-      <c r="AU57" s="26"/>
+      <c r="AL57" s="87"/>
+      <c r="AM57" s="88"/>
+      <c r="AN57" s="88"/>
+      <c r="AO57" s="88"/>
+      <c r="AP57" s="86"/>
+      <c r="AQ57" s="87"/>
+      <c r="AR57" s="88"/>
+      <c r="AS57" s="88"/>
+      <c r="AT57" s="88"/>
+      <c r="AU57" s="79" t="s">
+        <v>70</v>
+      </c>
       <c r="AY57" s="3"/>
       <c r="BD57" s="3"/>
       <c r="BH57" s="3"/>

</xml_diff>